<commit_message>
Generate Ltd Company packages from app/data and app/templates
Triggered by: 11cde9f44bf86074f86f061d458771bf8dd6c3db
</commit_message>
<xml_diff>
--- a/examples/ltd-latest/Financialaccounts.xlsx
+++ b/examples/ltd-latest/Financialaccounts.xlsx
@@ -7118,7 +7118,7 @@
       <sheetData sheetId="0">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>29600</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -7130,7 +7130,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>24400</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -7148,7 +7148,7 @@
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>137837</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -7211,7 +7211,7 @@
       <sheetData sheetId="1">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>19500</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -7223,7 +7223,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>14200</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -7241,7 +7241,7 @@
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>137586</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -7304,7 +7304,7 @@
       <sheetData sheetId="2">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>19900</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -7316,7 +7316,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>14900</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -7334,7 +7334,7 @@
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>137684</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -7397,7 +7397,7 @@
       <sheetData sheetId="3">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>19100</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -7409,7 +7409,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>14000</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -7427,7 +7427,7 @@
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>229588</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -7490,7 +7490,7 @@
       <sheetData sheetId="4">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>22200</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -7502,7 +7502,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>14600</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -7514,13 +7514,13 @@
             <v>0</v>
           </cell>
           <cell r="N1">
-            <v>0</v>
+            <v>2500</v>
           </cell>
           <cell r="O1">
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>91907</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -7583,7 +7583,7 @@
       <sheetData sheetId="5">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>18000</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -7595,7 +7595,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>13400</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -7613,7 +7613,7 @@
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>137960</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -7676,7 +7676,7 @@
       <sheetData sheetId="6">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>72400</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -7688,7 +7688,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>30400</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -7706,7 +7706,7 @@
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>230025</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -7769,7 +7769,7 @@
       <sheetData sheetId="7">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>19400</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -7781,7 +7781,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>14500</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -7799,7 +7799,7 @@
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>138138</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -7862,7 +7862,7 @@
       <sheetData sheetId="8">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>19100</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -7874,7 +7874,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>13900</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -7892,7 +7892,7 @@
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>184309</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -7955,7 +7955,7 @@
       <sheetData sheetId="9">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>27000</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -7967,7 +7967,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>15200</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -7979,13 +7979,13 @@
             <v>0</v>
           </cell>
           <cell r="N1">
-            <v>0</v>
+            <v>1500</v>
           </cell>
           <cell r="O1">
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>138305</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -8048,7 +8048,7 @@
       <sheetData sheetId="10">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>19700</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -8060,7 +8060,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>14300</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -8078,7 +8078,7 @@
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>92271</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -8141,7 +8141,7 @@
       <sheetData sheetId="11">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>24600</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -8153,7 +8153,7 @@
             <v>0</v>
           </cell>
           <cell r="J1">
-            <v>0</v>
+            <v>14800</v>
           </cell>
           <cell r="K1">
             <v>0</v>
@@ -8171,7 +8171,7 @@
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>184677</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -8722,7 +8722,7 @@
       <sheetData sheetId="5">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>125</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -8746,7 +8746,7 @@
             <v>0</v>
           </cell>
           <cell r="N1">
-            <v>0</v>
+            <v>125</v>
           </cell>
           <cell r="O1">
             <v>0</v>
@@ -9280,7 +9280,7 @@
       <sheetData sheetId="11">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>5150</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -9304,7 +9304,7 @@
             <v>0</v>
           </cell>
           <cell r="N1">
-            <v>0</v>
+            <v>150</v>
           </cell>
           <cell r="O1">
             <v>0</v>
@@ -9313,7 +9313,7 @@
             <v>0</v>
           </cell>
           <cell r="Q1">
-            <v>0</v>
+            <v>5000</v>
           </cell>
         </row>
         <row r="1">
@@ -9396,7 +9396,7 @@
       <sheetData sheetId="0">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>500</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -9429,7 +9429,7 @@
             <v>0</v>
           </cell>
           <cell r="Q1">
-            <v>0</v>
+            <v>500</v>
           </cell>
         </row>
         <row r="1">
@@ -9519,7 +9519,7 @@
             <v>0</v>
           </cell>
           <cell r="P1">
-            <v>0</v>
+            <v>45858</v>
           </cell>
           <cell r="Q1">
             <v>0</v>
@@ -9582,7 +9582,7 @@
       <sheetData sheetId="2">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>180</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -9675,7 +9675,7 @@
       <sheetData sheetId="3">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>300</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -9708,7 +9708,7 @@
             <v>0</v>
           </cell>
           <cell r="Q1">
-            <v>0</v>
+            <v>300</v>
           </cell>
         </row>
         <row r="1">
@@ -9954,7 +9954,7 @@
       <sheetData sheetId="6">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>620</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -9987,7 +9987,7 @@
             <v>0</v>
           </cell>
           <cell r="Q1">
-            <v>0</v>
+            <v>500</v>
           </cell>
         </row>
         <row r="1">
@@ -10233,7 +10233,7 @@
       <sheetData sheetId="9">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>300</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -10266,7 +10266,7 @@
             <v>0</v>
           </cell>
           <cell r="Q1">
-            <v>0</v>
+            <v>300</v>
           </cell>
         </row>
         <row r="1">
@@ -10326,7 +10326,7 @@
       <sheetData sheetId="10">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>240</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -10535,7 +10535,7 @@
       <sheetData sheetId="0">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>15</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -10697,7 +10697,7 @@
       <sheetData sheetId="2">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>125</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -10940,7 +10940,7 @@
       <sheetData sheetId="5">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>18</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -11183,7 +11183,7 @@
       <sheetData sheetId="8">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>50</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -11426,7 +11426,7 @@
       <sheetData sheetId="11">
         <row r="1">
           <cell r="F1">
-            <v>0</v>
+            <v>12</v>
           </cell>
           <cell r="G1">
             <v>0</v>
@@ -21386,7 +21386,7 @@
       <c r="G20" s="36"/>
       <c r="H20" s="36" t="n">
         <f aca="false">-[4]Jun!$J$1</f>
-        <v>-0</v>
+        <v>-24400</v>
       </c>
       <c r="I20" s="36" t="n">
         <f aca="false">-[5]Jun!$J$1</f>
@@ -21404,7 +21404,7 @@
       <c r="N20" s="57"/>
       <c r="O20" s="36" t="n">
         <f aca="false">SUM(D20:N20)</f>
-        <v>33400</v>
+        <v>9000</v>
       </c>
       <c r="P20" s="57"/>
       <c r="Q20" s="36" t="n">
@@ -21414,7 +21414,7 @@
       <c r="R20" s="36"/>
       <c r="S20" s="36" t="n">
         <f aca="false">-[4]Jul!$J$1</f>
-        <v>-0</v>
+        <v>-14200</v>
       </c>
       <c r="T20" s="36" t="n">
         <f aca="false">-[5]Jul!$J$1</f>
@@ -21435,7 +21435,7 @@
       <c r="Y20" s="54"/>
       <c r="Z20" s="36" t="n">
         <f aca="false">SUM(O20:Y20)</f>
-        <v>66320</v>
+        <v>27720</v>
       </c>
       <c r="AA20" s="57"/>
       <c r="AB20" s="36" t="n">
@@ -21445,7 +21445,7 @@
       <c r="AC20" s="36"/>
       <c r="AD20" s="36" t="n">
         <f aca="false">-[4]Aug!$J$1</f>
-        <v>-0</v>
+        <v>-14900</v>
       </c>
       <c r="AE20" s="36" t="n">
         <f aca="false">-[5]Aug!$J$1</f>
@@ -21464,7 +21464,7 @@
       <c r="AJ20" s="54"/>
       <c r="AK20" s="36" t="n">
         <f aca="false">SUM(Z20:AJ20)</f>
-        <v>101520</v>
+        <v>48020</v>
       </c>
       <c r="AL20" s="57"/>
       <c r="AM20" s="36" t="n">
@@ -21474,7 +21474,7 @@
       <c r="AN20" s="36"/>
       <c r="AO20" s="36" t="n">
         <f aca="false">-[4]Sep!$J$1</f>
-        <v>-0</v>
+        <v>-14000</v>
       </c>
       <c r="AP20" s="36" t="n">
         <f aca="false">-[5]Sep!$J$1</f>
@@ -21493,7 +21493,7 @@
       <c r="AU20" s="54"/>
       <c r="AV20" s="36" t="n">
         <f aca="false">SUM(AK20:AU20)</f>
-        <v>135280</v>
+        <v>67780</v>
       </c>
       <c r="AW20" s="57"/>
       <c r="AX20" s="36" t="n">
@@ -21503,7 +21503,7 @@
       <c r="AY20" s="36"/>
       <c r="AZ20" s="36" t="n">
         <f aca="false">-[4]Oct!$J$1</f>
-        <v>-0</v>
+        <v>-14600</v>
       </c>
       <c r="BA20" s="36" t="n">
         <f aca="false">-[5]Oct!$J$1</f>
@@ -21522,7 +21522,7 @@
       <c r="BF20" s="54"/>
       <c r="BG20" s="36" t="n">
         <f aca="false">SUM(AV20:BF20)</f>
-        <v>171300</v>
+        <v>89200</v>
       </c>
       <c r="BH20" s="57"/>
       <c r="BI20" s="36" t="n">
@@ -21532,7 +21532,7 @@
       <c r="BJ20" s="36"/>
       <c r="BK20" s="36" t="n">
         <f aca="false">-[4]Nov!$J$1</f>
-        <v>-0</v>
+        <v>-13400</v>
       </c>
       <c r="BL20" s="36" t="n">
         <f aca="false">-[5]Nov!$J$1</f>
@@ -21551,7 +21551,7 @@
       <c r="BQ20" s="54"/>
       <c r="BR20" s="36" t="n">
         <f aca="false">SUM(BG20:BQ20)</f>
-        <v>205060</v>
+        <v>109560</v>
       </c>
       <c r="BS20" s="57"/>
       <c r="BT20" s="36" t="n">
@@ -21561,7 +21561,7 @@
       <c r="BU20" s="36"/>
       <c r="BV20" s="36" t="n">
         <f aca="false">-[4]Dec!$J$1</f>
-        <v>-0</v>
+        <v>-30400</v>
       </c>
       <c r="BW20" s="36" t="n">
         <f aca="false">-[5]Dec!$J$1</f>
@@ -21580,7 +21580,7 @@
       <c r="CB20" s="54"/>
       <c r="CC20" s="36" t="n">
         <f aca="false">SUM(BR20:CB20)</f>
-        <v>255620</v>
+        <v>129720</v>
       </c>
       <c r="CD20" s="57"/>
       <c r="CE20" s="36" t="n">
@@ -21590,7 +21590,7 @@
       <c r="CF20" s="36"/>
       <c r="CG20" s="36" t="n">
         <f aca="false">-[4]Jan!$J$1</f>
-        <v>-0</v>
+        <v>-14500</v>
       </c>
       <c r="CH20" s="36" t="n">
         <f aca="false">-[5]Jan!$J$1</f>
@@ -21609,7 +21609,7 @@
       <c r="CM20" s="54"/>
       <c r="CN20" s="36" t="n">
         <f aca="false">SUM(CC20:CM20)</f>
-        <v>290940</v>
+        <v>150540</v>
       </c>
       <c r="CO20" s="57"/>
       <c r="CP20" s="36" t="n">
@@ -21619,7 +21619,7 @@
       <c r="CQ20" s="36"/>
       <c r="CR20" s="36" t="n">
         <f aca="false">-[4]Feb!$J$1</f>
-        <v>-0</v>
+        <v>-13900</v>
       </c>
       <c r="CS20" s="36" t="n">
         <f aca="false">-[5]Feb!$J$1</f>
@@ -21638,7 +21638,7 @@
       <c r="CX20" s="54"/>
       <c r="CY20" s="36" t="n">
         <f aca="false">SUM(CN20:CX20)</f>
-        <v>323740</v>
+        <v>169440</v>
       </c>
       <c r="CZ20" s="57"/>
       <c r="DA20" s="36" t="n">
@@ -21648,7 +21648,7 @@
       <c r="DB20" s="36"/>
       <c r="DC20" s="36" t="n">
         <f aca="false">-[4]Mar!$J$1</f>
-        <v>-0</v>
+        <v>-15200</v>
       </c>
       <c r="DD20" s="36" t="n">
         <f aca="false">-[5]Mar!$J$1</f>
@@ -21667,7 +21667,7 @@
       <c r="DI20" s="54"/>
       <c r="DJ20" s="36" t="n">
         <f aca="false">SUM(CY20:DI20)</f>
-        <v>359180</v>
+        <v>189680</v>
       </c>
       <c r="DK20" s="57"/>
       <c r="DL20" s="36" t="n">
@@ -21677,7 +21677,7 @@
       <c r="DM20" s="36"/>
       <c r="DN20" s="36" t="n">
         <f aca="false">-[4]Apr!$J$1</f>
-        <v>-0</v>
+        <v>-14300</v>
       </c>
       <c r="DO20" s="36" t="n">
         <f aca="false">-[5]Apr!$J$1</f>
@@ -21696,7 +21696,7 @@
       <c r="DT20" s="54"/>
       <c r="DU20" s="36" t="n">
         <f aca="false">SUM(DJ20:DT20)</f>
-        <v>393540</v>
+        <v>209740</v>
       </c>
       <c r="DV20" s="57"/>
       <c r="DW20" s="36" t="n">
@@ -21706,7 +21706,7 @@
       <c r="DX20" s="36"/>
       <c r="DY20" s="36" t="n">
         <f aca="false">-[4]May!$J$1</f>
-        <v>-0</v>
+        <v>-14800</v>
       </c>
       <c r="DZ20" s="36" t="n">
         <f aca="false">-[5]May!$J$1</f>
@@ -21725,13 +21725,13 @@
       <c r="EE20" s="54"/>
       <c r="EF20" s="36" t="n">
         <f aca="false">SUM(DU20:EE20)</f>
-        <v>424900</v>
+        <v>226300</v>
       </c>
       <c r="EG20" s="54"/>
       <c r="EI20" s="54"/>
       <c r="EJ20" s="36" t="n">
         <f aca="false">SUM(EF20:EH20)</f>
-        <v>424900</v>
+        <v>226300</v>
       </c>
       <c r="EK20" s="54"/>
     </row>
@@ -21888,7 +21888,7 @@
       <c r="G22" s="36"/>
       <c r="H22" s="36" t="n">
         <f aca="false">[4]Jun!$F$1-[4]Jun!$X$1</f>
-        <v>0</v>
+        <v>29600</v>
       </c>
       <c r="I22" s="36"/>
       <c r="J22" s="36"/>
@@ -21897,14 +21897,14 @@
       <c r="N22" s="57"/>
       <c r="O22" s="36" t="n">
         <f aca="false">SUM(D22:N22)</f>
-        <v>0</v>
+        <v>29600</v>
       </c>
       <c r="P22" s="57"/>
       <c r="Q22" s="36"/>
       <c r="R22" s="36"/>
       <c r="S22" s="36" t="n">
         <f aca="false">[4]Jul!$F$1-[4]Jul!$X$1</f>
-        <v>0</v>
+        <v>19500</v>
       </c>
       <c r="T22" s="36"/>
       <c r="U22" s="36"/>
@@ -21914,14 +21914,14 @@
       <c r="Y22" s="54"/>
       <c r="Z22" s="36" t="n">
         <f aca="false">SUM(O22:Y22)</f>
-        <v>0</v>
+        <v>49100</v>
       </c>
       <c r="AA22" s="57"/>
       <c r="AB22" s="36"/>
       <c r="AC22" s="36"/>
       <c r="AD22" s="36" t="n">
         <f aca="false">[4]Aug!$F$1-[4]Aug!$X$1</f>
-        <v>0</v>
+        <v>19900</v>
       </c>
       <c r="AE22" s="36"/>
       <c r="AF22" s="36"/>
@@ -21931,14 +21931,14 @@
       <c r="AJ22" s="54"/>
       <c r="AK22" s="36" t="n">
         <f aca="false">SUM(Z22:AJ22)</f>
-        <v>0</v>
+        <v>69000</v>
       </c>
       <c r="AL22" s="57"/>
       <c r="AM22" s="36"/>
       <c r="AN22" s="36"/>
       <c r="AO22" s="36" t="n">
         <f aca="false">[4]Sep!$F$1-[4]Sep!$X$1</f>
-        <v>0</v>
+        <v>19100</v>
       </c>
       <c r="AP22" s="36"/>
       <c r="AQ22" s="36"/>
@@ -21948,14 +21948,14 @@
       <c r="AU22" s="54"/>
       <c r="AV22" s="36" t="n">
         <f aca="false">SUM(AK22:AU22)</f>
-        <v>0</v>
+        <v>88100</v>
       </c>
       <c r="AW22" s="57"/>
       <c r="AX22" s="36"/>
       <c r="AY22" s="36"/>
       <c r="AZ22" s="36" t="n">
         <f aca="false">[4]Oct!$F$1-[4]Oct!$X$1</f>
-        <v>0</v>
+        <v>22200</v>
       </c>
       <c r="BA22" s="36"/>
       <c r="BB22" s="36"/>
@@ -21965,14 +21965,14 @@
       <c r="BF22" s="54"/>
       <c r="BG22" s="36" t="n">
         <f aca="false">SUM(AV22:BF22)</f>
-        <v>0</v>
+        <v>110300</v>
       </c>
       <c r="BH22" s="57"/>
       <c r="BI22" s="36"/>
       <c r="BJ22" s="36"/>
       <c r="BK22" s="36" t="n">
         <f aca="false">[4]Nov!$F$1-[4]Nov!$X$1</f>
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="BL22" s="36"/>
       <c r="BM22" s="36"/>
@@ -21982,14 +21982,14 @@
       <c r="BQ22" s="54"/>
       <c r="BR22" s="36" t="n">
         <f aca="false">SUM(BG22:BQ22)</f>
-        <v>0</v>
+        <v>128300</v>
       </c>
       <c r="BS22" s="57"/>
       <c r="BT22" s="36"/>
       <c r="BU22" s="36"/>
       <c r="BV22" s="36" t="n">
         <f aca="false">[4]Dec!$F$1-[4]Dec!$X$1</f>
-        <v>0</v>
+        <v>72400</v>
       </c>
       <c r="BW22" s="36"/>
       <c r="BX22" s="36"/>
@@ -21999,14 +21999,14 @@
       <c r="CB22" s="54"/>
       <c r="CC22" s="36" t="n">
         <f aca="false">SUM(BR22:CB22)</f>
-        <v>0</v>
+        <v>200700</v>
       </c>
       <c r="CD22" s="57"/>
       <c r="CE22" s="36"/>
       <c r="CF22" s="36"/>
       <c r="CG22" s="36" t="n">
         <f aca="false">[4]Jan!$F$1-[4]Jan!$X$1</f>
-        <v>0</v>
+        <v>19400</v>
       </c>
       <c r="CH22" s="36"/>
       <c r="CI22" s="36"/>
@@ -22016,14 +22016,14 @@
       <c r="CM22" s="54"/>
       <c r="CN22" s="36" t="n">
         <f aca="false">SUM(CC22:CM22)</f>
-        <v>0</v>
+        <v>220100</v>
       </c>
       <c r="CO22" s="57"/>
       <c r="CP22" s="36"/>
       <c r="CQ22" s="36"/>
       <c r="CR22" s="36" t="n">
         <f aca="false">[4]Feb!$F$1-[4]Feb!$X$1</f>
-        <v>0</v>
+        <v>19100</v>
       </c>
       <c r="CS22" s="36"/>
       <c r="CT22" s="36"/>
@@ -22033,14 +22033,14 @@
       <c r="CX22" s="54"/>
       <c r="CY22" s="36" t="n">
         <f aca="false">SUM(CN22:CX22)</f>
-        <v>0</v>
+        <v>239200</v>
       </c>
       <c r="CZ22" s="57"/>
       <c r="DA22" s="36"/>
       <c r="DB22" s="36"/>
       <c r="DC22" s="36" t="n">
         <f aca="false">[4]Mar!$F$1-[4]Mar!$X$1</f>
-        <v>0</v>
+        <v>27000</v>
       </c>
       <c r="DD22" s="36"/>
       <c r="DE22" s="36"/>
@@ -22050,14 +22050,14 @@
       <c r="DI22" s="54"/>
       <c r="DJ22" s="36" t="n">
         <f aca="false">SUM(CY22:DI22)</f>
-        <v>0</v>
+        <v>266200</v>
       </c>
       <c r="DK22" s="57"/>
       <c r="DL22" s="36"/>
       <c r="DM22" s="36"/>
       <c r="DN22" s="36" t="n">
         <f aca="false">[4]Apr!$F$1-[4]Apr!$X$1</f>
-        <v>0</v>
+        <v>19700</v>
       </c>
       <c r="DO22" s="36"/>
       <c r="DP22" s="36"/>
@@ -22067,14 +22067,14 @@
       <c r="DT22" s="54"/>
       <c r="DU22" s="36" t="n">
         <f aca="false">SUM(DJ22:DT22)</f>
-        <v>0</v>
+        <v>285900</v>
       </c>
       <c r="DV22" s="57"/>
       <c r="DW22" s="36"/>
       <c r="DX22" s="36"/>
       <c r="DY22" s="36" t="n">
         <f aca="false">[4]May!$F$1-[4]May!$X$1</f>
-        <v>0</v>
+        <v>24600</v>
       </c>
       <c r="DZ22" s="36"/>
       <c r="EA22" s="36"/>
@@ -22084,13 +22084,13 @@
       <c r="EE22" s="54"/>
       <c r="EF22" s="36" t="n">
         <f aca="false">SUM(DU22:EE22)</f>
-        <v>0</v>
+        <v>310500</v>
       </c>
       <c r="EG22" s="54"/>
       <c r="EI22" s="54"/>
       <c r="EJ22" s="36" t="n">
         <f aca="false">SUM(EF22:EH22)</f>
-        <v>0</v>
+        <v>310500</v>
       </c>
       <c r="EK22" s="54"/>
     </row>
@@ -22196,7 +22196,7 @@
       <c r="BK23" s="36"/>
       <c r="BL23" s="36" t="n">
         <f aca="false">[5]Nov!$F$1-[5]Nov!$X$1</f>
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="BM23" s="36"/>
       <c r="BN23" s="36"/>
@@ -22205,7 +22205,7 @@
       <c r="BQ23" s="54"/>
       <c r="BR23" s="36" t="n">
         <f aca="false">SUM(BG23:BQ23)</f>
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="BS23" s="57"/>
       <c r="BT23" s="36"/>
@@ -22222,7 +22222,7 @@
       <c r="CB23" s="54"/>
       <c r="CC23" s="36" t="n">
         <f aca="false">SUM(BR23:CB23)</f>
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="CD23" s="57"/>
       <c r="CE23" s="36"/>
@@ -22239,7 +22239,7 @@
       <c r="CM23" s="54"/>
       <c r="CN23" s="36" t="n">
         <f aca="false">SUM(CC23:CM23)</f>
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="CO23" s="57"/>
       <c r="CP23" s="36"/>
@@ -22256,7 +22256,7 @@
       <c r="CX23" s="54"/>
       <c r="CY23" s="36" t="n">
         <f aca="false">SUM(CN23:CX23)</f>
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="CZ23" s="57"/>
       <c r="DA23" s="36"/>
@@ -22273,7 +22273,7 @@
       <c r="DI23" s="54"/>
       <c r="DJ23" s="36" t="n">
         <f aca="false">SUM(CY23:DI23)</f>
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="DK23" s="57"/>
       <c r="DL23" s="36"/>
@@ -22290,7 +22290,7 @@
       <c r="DT23" s="54"/>
       <c r="DU23" s="36" t="n">
         <f aca="false">SUM(DJ23:DT23)</f>
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="DV23" s="57"/>
       <c r="DW23" s="36"/>
@@ -22298,7 +22298,7 @@
       <c r="DY23" s="36"/>
       <c r="DZ23" s="36" t="n">
         <f aca="false">[5]May!$F$1-[5]May!$X$1</f>
-        <v>0</v>
+        <v>5150</v>
       </c>
       <c r="EA23" s="36"/>
       <c r="EB23" s="36"/>
@@ -22307,13 +22307,13 @@
       <c r="EE23" s="54"/>
       <c r="EF23" s="36" t="n">
         <f aca="false">SUM(DU23:EE23)</f>
-        <v>0</v>
+        <v>5275</v>
       </c>
       <c r="EG23" s="54"/>
       <c r="EI23" s="54"/>
       <c r="EJ23" s="36" t="n">
         <f aca="false">SUM(EF23:EH23)</f>
-        <v>0</v>
+        <v>5275</v>
       </c>
       <c r="EK23" s="54"/>
     </row>
@@ -22336,14 +22336,14 @@
       <c r="I24" s="36"/>
       <c r="J24" s="36" t="n">
         <f aca="false">[6]Jun!$F$1-[6]Jun!$X$1</f>
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="K24" s="36"/>
       <c r="L24" s="36"/>
       <c r="N24" s="57"/>
       <c r="O24" s="36" t="n">
         <f aca="false">SUM(D24:N24)</f>
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="P24" s="57"/>
       <c r="Q24" s="36"/>
@@ -22360,7 +22360,7 @@
       <c r="Y24" s="54"/>
       <c r="Z24" s="36" t="n">
         <f aca="false">SUM(O24:Y24)</f>
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="AA24" s="57"/>
       <c r="AB24" s="36"/>
@@ -22369,7 +22369,7 @@
       <c r="AE24" s="36"/>
       <c r="AF24" s="36" t="n">
         <f aca="false">[6]Aug!$F$1-[6]Aug!$X$1</f>
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="AG24" s="36"/>
       <c r="AH24" s="36"/>
@@ -22377,7 +22377,7 @@
       <c r="AJ24" s="54"/>
       <c r="AK24" s="36" t="n">
         <f aca="false">SUM(Z24:AJ24)</f>
-        <v>0</v>
+        <v>680</v>
       </c>
       <c r="AL24" s="57"/>
       <c r="AM24" s="36"/>
@@ -22386,7 +22386,7 @@
       <c r="AP24" s="36"/>
       <c r="AQ24" s="36" t="n">
         <f aca="false">[6]Sep!$F$1-[6]Sep!$X$1</f>
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="AR24" s="36"/>
       <c r="AS24" s="36"/>
@@ -22394,7 +22394,7 @@
       <c r="AU24" s="54"/>
       <c r="AV24" s="36" t="n">
         <f aca="false">SUM(AK24:AU24)</f>
-        <v>0</v>
+        <v>980</v>
       </c>
       <c r="AW24" s="57"/>
       <c r="AX24" s="36"/>
@@ -22411,7 +22411,7 @@
       <c r="BF24" s="54"/>
       <c r="BG24" s="36" t="n">
         <f aca="false">SUM(AV24:BF24)</f>
-        <v>0</v>
+        <v>980</v>
       </c>
       <c r="BH24" s="57"/>
       <c r="BI24" s="36"/>
@@ -22428,7 +22428,7 @@
       <c r="BQ24" s="54"/>
       <c r="BR24" s="36" t="n">
         <f aca="false">SUM(BG24:BQ24)</f>
-        <v>0</v>
+        <v>980</v>
       </c>
       <c r="BS24" s="57"/>
       <c r="BT24" s="36"/>
@@ -22437,7 +22437,7 @@
       <c r="BW24" s="36"/>
       <c r="BX24" s="36" t="n">
         <f aca="false">[6]Dec!$F$1-[6]Dec!$X$1</f>
-        <v>0</v>
+        <v>620</v>
       </c>
       <c r="BY24" s="36"/>
       <c r="BZ24" s="36"/>
@@ -22445,7 +22445,7 @@
       <c r="CB24" s="54"/>
       <c r="CC24" s="36" t="n">
         <f aca="false">SUM(BR24:CB24)</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="CD24" s="57"/>
       <c r="CE24" s="36"/>
@@ -22462,7 +22462,7 @@
       <c r="CM24" s="54"/>
       <c r="CN24" s="36" t="n">
         <f aca="false">SUM(CC24:CM24)</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="CO24" s="57"/>
       <c r="CP24" s="36"/>
@@ -22479,7 +22479,7 @@
       <c r="CX24" s="54"/>
       <c r="CY24" s="36" t="n">
         <f aca="false">SUM(CN24:CX24)</f>
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="CZ24" s="57"/>
       <c r="DA24" s="36"/>
@@ -22488,7 +22488,7 @@
       <c r="DD24" s="36"/>
       <c r="DE24" s="36" t="n">
         <f aca="false">[6]Mar!$F$1-[6]Mar!$X$1</f>
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="DF24" s="36"/>
       <c r="DG24" s="36"/>
@@ -22496,7 +22496,7 @@
       <c r="DI24" s="54"/>
       <c r="DJ24" s="36" t="n">
         <f aca="false">SUM(CY24:DI24)</f>
-        <v>0</v>
+        <v>1900</v>
       </c>
       <c r="DK24" s="57"/>
       <c r="DL24" s="36"/>
@@ -22505,7 +22505,7 @@
       <c r="DO24" s="36"/>
       <c r="DP24" s="36" t="n">
         <f aca="false">[6]Apr!$F$1-[6]Apr!$X$1</f>
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="DQ24" s="36"/>
       <c r="DR24" s="36"/>
@@ -22513,7 +22513,7 @@
       <c r="DT24" s="54"/>
       <c r="DU24" s="36" t="n">
         <f aca="false">SUM(DJ24:DT24)</f>
-        <v>0</v>
+        <v>2140</v>
       </c>
       <c r="DV24" s="57"/>
       <c r="DW24" s="36"/>
@@ -22530,13 +22530,13 @@
       <c r="EE24" s="54"/>
       <c r="EF24" s="36" t="n">
         <f aca="false">SUM(DU24:EE24)</f>
-        <v>0</v>
+        <v>2140</v>
       </c>
       <c r="EG24" s="54"/>
       <c r="EI24" s="54"/>
       <c r="EJ24" s="36" t="n">
         <f aca="false">SUM(EF24:EH24)</f>
-        <v>0</v>
+        <v>2140</v>
       </c>
       <c r="EK24" s="54"/>
     </row>
@@ -22560,13 +22560,13 @@
       <c r="J25" s="36"/>
       <c r="K25" s="36" t="n">
         <f aca="false">[7]Jun!$F$1-[7]Jun!$U$1</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="L25" s="36"/>
       <c r="N25" s="57"/>
       <c r="O25" s="36" t="n">
         <f aca="false">SUM(D25:N25)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="P25" s="57"/>
       <c r="Q25" s="36"/>
@@ -22583,7 +22583,7 @@
       <c r="Y25" s="54"/>
       <c r="Z25" s="36" t="n">
         <f aca="false">SUM(O25:Y25)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="AA25" s="57"/>
       <c r="AB25" s="36"/>
@@ -22593,14 +22593,14 @@
       <c r="AF25" s="36"/>
       <c r="AG25" s="36" t="n">
         <f aca="false">[7]Aug!$F$1-[7]Aug!$U$1</f>
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="AH25" s="36"/>
       <c r="AI25" s="36"/>
       <c r="AJ25" s="54"/>
       <c r="AK25" s="36" t="n">
         <f aca="false">SUM(Z25:AJ25)</f>
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="AL25" s="57"/>
       <c r="AM25" s="36"/>
@@ -22617,7 +22617,7 @@
       <c r="AU25" s="54"/>
       <c r="AV25" s="36" t="n">
         <f aca="false">SUM(AK25:AU25)</f>
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="AW25" s="57"/>
       <c r="AX25" s="36"/>
@@ -22634,7 +22634,7 @@
       <c r="BF25" s="54"/>
       <c r="BG25" s="36" t="n">
         <f aca="false">SUM(AV25:BF25)</f>
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="BH25" s="57"/>
       <c r="BI25" s="36"/>
@@ -22644,14 +22644,14 @@
       <c r="BM25" s="36"/>
       <c r="BN25" s="36" t="n">
         <f aca="false">[7]Nov!$F$1-[7]Nov!$U$1</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="BO25" s="36"/>
       <c r="BP25" s="36"/>
       <c r="BQ25" s="54"/>
       <c r="BR25" s="36" t="n">
         <f aca="false">SUM(BG25:BQ25)</f>
-        <v>0</v>
+        <v>158</v>
       </c>
       <c r="BS25" s="57"/>
       <c r="BT25" s="36"/>
@@ -22668,7 +22668,7 @@
       <c r="CB25" s="54"/>
       <c r="CC25" s="36" t="n">
         <f aca="false">SUM(BR25:CB25)</f>
-        <v>0</v>
+        <v>158</v>
       </c>
       <c r="CD25" s="57"/>
       <c r="CE25" s="36"/>
@@ -22685,7 +22685,7 @@
       <c r="CM25" s="54"/>
       <c r="CN25" s="36" t="n">
         <f aca="false">SUM(CC25:CM25)</f>
-        <v>0</v>
+        <v>158</v>
       </c>
       <c r="CO25" s="57"/>
       <c r="CP25" s="36"/>
@@ -22695,14 +22695,14 @@
       <c r="CT25" s="36"/>
       <c r="CU25" s="36" t="n">
         <f aca="false">[7]Feb!$F$1-[7]Feb!$U$1</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="CV25" s="36"/>
       <c r="CW25" s="36"/>
       <c r="CX25" s="54"/>
       <c r="CY25" s="36" t="n">
         <f aca="false">SUM(CN25:CX25)</f>
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="CZ25" s="57"/>
       <c r="DA25" s="36"/>
@@ -22719,7 +22719,7 @@
       <c r="DI25" s="54"/>
       <c r="DJ25" s="36" t="n">
         <f aca="false">SUM(CY25:DI25)</f>
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="DK25" s="57"/>
       <c r="DL25" s="36"/>
@@ -22736,7 +22736,7 @@
       <c r="DT25" s="54"/>
       <c r="DU25" s="36" t="n">
         <f aca="false">SUM(DJ25:DT25)</f>
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="DV25" s="57"/>
       <c r="DW25" s="36"/>
@@ -22746,14 +22746,14 @@
       <c r="EA25" s="36"/>
       <c r="EB25" s="36" t="n">
         <f aca="false">[7]May!$F$1-[7]May!$U$1</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="EC25" s="36"/>
       <c r="ED25" s="36"/>
       <c r="EE25" s="54"/>
       <c r="EF25" s="36" t="n">
         <f aca="false">SUM(DU25:EE25)</f>
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="EG25" s="54"/>
       <c r="EH25" s="36" t="n">
@@ -22763,7 +22763,7 @@
       <c r="EI25" s="54"/>
       <c r="EJ25" s="36" t="n">
         <f aca="false">SUM(EF25:EH25)</f>
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="EK25" s="54"/>
     </row>
@@ -25076,7 +25076,7 @@
       </c>
       <c r="AZ33" s="36" t="n">
         <f aca="false">-[4]Oct!$N$1+[4]Oct!$AI$1</f>
-        <v>0</v>
+        <v>-2500</v>
       </c>
       <c r="BA33" s="36" t="n">
         <f aca="false">-[5]Oct!$N$1+[5]Oct!$AI$1</f>
@@ -25095,7 +25095,7 @@
       <c r="BF33" s="54"/>
       <c r="BG33" s="36" t="n">
         <f aca="false">SUM(AV33:BF33)</f>
-        <v>-28550</v>
+        <v>-31050</v>
       </c>
       <c r="BH33" s="57"/>
       <c r="BI33" s="36" t="n">
@@ -25112,7 +25112,7 @@
       </c>
       <c r="BL33" s="36" t="n">
         <f aca="false">-[5]Nov!$N$1+[5]Nov!$AI$1</f>
-        <v>0</v>
+        <v>-125</v>
       </c>
       <c r="BM33" s="36" t="n">
         <f aca="false">-[6]Nov!$N$1+[6]Nov!$AI$1</f>
@@ -25127,7 +25127,7 @@
       <c r="BQ33" s="54"/>
       <c r="BR33" s="36" t="n">
         <f aca="false">SUM(BG33:BQ33)</f>
-        <v>-34176.6666666667</v>
+        <v>-36801.6666666667</v>
       </c>
       <c r="BS33" s="57"/>
       <c r="BT33" s="36" t="n">
@@ -25159,7 +25159,7 @@
       <c r="CB33" s="54"/>
       <c r="CC33" s="36" t="n">
         <f aca="false">SUM(BR33:CB33)</f>
-        <v>-42603.3333333334</v>
+        <v>-45228.3333333334</v>
       </c>
       <c r="CD33" s="57"/>
       <c r="CE33" s="36" t="n">
@@ -25191,7 +25191,7 @@
       <c r="CM33" s="54"/>
       <c r="CN33" s="36" t="n">
         <f aca="false">SUM(CC33:CM33)</f>
-        <v>-48490</v>
+        <v>-51115</v>
       </c>
       <c r="CO33" s="57"/>
       <c r="CP33" s="36" t="n">
@@ -25223,7 +25223,7 @@
       <c r="CX33" s="54"/>
       <c r="CY33" s="36" t="n">
         <f aca="false">SUM(CN33:CX33)</f>
-        <v>-53956.6666666667</v>
+        <v>-56581.6666666667</v>
       </c>
       <c r="CZ33" s="57"/>
       <c r="DA33" s="36" t="n">
@@ -25236,7 +25236,7 @@
       </c>
       <c r="DC33" s="36" t="n">
         <f aca="false">-[4]Mar!$N$1+[4]Mar!$AI$1</f>
-        <v>0</v>
+        <v>-1500</v>
       </c>
       <c r="DD33" s="36" t="n">
         <f aca="false">-[5]Mar!$N$1+[5]Mar!$AI$1</f>
@@ -25255,7 +25255,7 @@
       <c r="DI33" s="54"/>
       <c r="DJ33" s="36" t="n">
         <f aca="false">SUM(CY33:DI33)</f>
-        <v>-59863.3333333334</v>
+        <v>-63988.3333333334</v>
       </c>
       <c r="DK33" s="57"/>
       <c r="DL33" s="36" t="n">
@@ -25287,7 +25287,7 @@
       <c r="DT33" s="54"/>
       <c r="DU33" s="36" t="n">
         <f aca="false">SUM(DJ33:DT33)</f>
-        <v>-65590</v>
+        <v>-69715</v>
       </c>
       <c r="DV33" s="57"/>
       <c r="DW33" s="36" t="n">
@@ -25304,7 +25304,7 @@
       </c>
       <c r="DZ33" s="36" t="n">
         <f aca="false">-[5]May!$N$1+[5]May!$AI$1</f>
-        <v>0</v>
+        <v>-150</v>
       </c>
       <c r="EA33" s="36" t="n">
         <f aca="false">-[6]May!$N$1+[6]May!$AI$1</f>
@@ -25319,13 +25319,13 @@
       <c r="EE33" s="54"/>
       <c r="EF33" s="36" t="n">
         <f aca="false">SUM(DU33:EE33)</f>
-        <v>-70816.6666666667</v>
+        <v>-75091.6666666667</v>
       </c>
       <c r="EG33" s="54"/>
       <c r="EI33" s="54"/>
       <c r="EJ33" s="36" t="n">
         <f aca="false">SUM(EF33:EH33)</f>
-        <v>-70816.6666666667</v>
+        <v>-75091.6666666667</v>
       </c>
       <c r="EK33" s="54"/>
     </row>
@@ -26015,12 +26015,12 @@
       <c r="EC35" s="36"/>
       <c r="ED35" s="36" t="n">
         <f aca="false">-CorporationTax!K35</f>
-        <v>-51792.3058333333</v>
+        <v>-53046.3058333333</v>
       </c>
       <c r="EE35" s="54"/>
       <c r="EF35" s="36" t="n">
         <f aca="false">SUM(DU35:EE35)</f>
-        <v>-51792.3058333333</v>
+        <v>-53046.3058333333</v>
       </c>
       <c r="EG35" s="54"/>
       <c r="EH35" s="36" t="n">
@@ -26030,7 +26030,7 @@
       <c r="EI35" s="54"/>
       <c r="EJ35" s="36" t="n">
         <f aca="false">SUM(EF35:EH35)</f>
-        <v>-51792.3058333333</v>
+        <v>-53046.3058333333</v>
       </c>
       <c r="EK35" s="54"/>
     </row>
@@ -26654,7 +26654,7 @@
       <c r="G39" s="36"/>
       <c r="H39" s="36" t="n">
         <f aca="false">-[4]Jun!$P$1+[4]Jun!$AM$1</f>
-        <v>0</v>
+        <v>-137837</v>
       </c>
       <c r="I39" s="36" t="n">
         <f aca="false">-[5]Jun!$P$1+[5]Jun!$AM$1</f>
@@ -26672,14 +26672,14 @@
       <c r="N39" s="57"/>
       <c r="O39" s="36" t="n">
         <f aca="false">SUM(D39:N39)</f>
-        <v>0</v>
+        <v>-137837</v>
       </c>
       <c r="P39" s="57"/>
       <c r="Q39" s="36"/>
       <c r="R39" s="36"/>
       <c r="S39" s="36" t="n">
         <f aca="false">-[4]Jul!$P$1+[4]Jul!$AM$1</f>
-        <v>0</v>
+        <v>-137586</v>
       </c>
       <c r="T39" s="36" t="n">
         <f aca="false">-[5]Jul!$P$1+[5]Jul!$AM$1</f>
@@ -26687,7 +26687,7 @@
       </c>
       <c r="U39" s="36" t="n">
         <f aca="false">-[6]Jul!$P$1+[6]Jul!$AM$1</f>
-        <v>0</v>
+        <v>-45858</v>
       </c>
       <c r="V39" s="36" t="n">
         <f aca="false">-[7]Jul!$N$1+[7]Jul!$AJ$1</f>
@@ -26698,14 +26698,14 @@
       <c r="Y39" s="54"/>
       <c r="Z39" s="36" t="n">
         <f aca="false">SUM(O39:Y39)</f>
-        <v>0</v>
+        <v>-321281</v>
       </c>
       <c r="AA39" s="57"/>
       <c r="AB39" s="36"/>
       <c r="AC39" s="36"/>
       <c r="AD39" s="36" t="n">
         <f aca="false">-[4]Aug!$P$1+[4]Aug!$AM$1</f>
-        <v>0</v>
+        <v>-137684</v>
       </c>
       <c r="AE39" s="36" t="n">
         <f aca="false">-[5]Aug!$P$1+[5]Aug!$AM$1</f>
@@ -26724,14 +26724,14 @@
       <c r="AJ39" s="54"/>
       <c r="AK39" s="36" t="n">
         <f aca="false">SUM(Z39:AJ39)</f>
-        <v>0</v>
+        <v>-458965</v>
       </c>
       <c r="AL39" s="57"/>
       <c r="AM39" s="36"/>
       <c r="AN39" s="36"/>
       <c r="AO39" s="36" t="n">
         <f aca="false">-[4]Sep!$P$1+[4]Sep!$AM$1</f>
-        <v>0</v>
+        <v>-229588</v>
       </c>
       <c r="AP39" s="36" t="n">
         <f aca="false">-[5]Sep!$P$1+[5]Sep!$AM$1</f>
@@ -26750,14 +26750,14 @@
       <c r="AU39" s="54"/>
       <c r="AV39" s="36" t="n">
         <f aca="false">SUM(AK39:AU39)</f>
-        <v>0</v>
+        <v>-688553</v>
       </c>
       <c r="AW39" s="57"/>
       <c r="AX39" s="36"/>
       <c r="AY39" s="36"/>
       <c r="AZ39" s="36" t="n">
         <f aca="false">-[4]Oct!$P$1+[4]Oct!$AM$1</f>
-        <v>0</v>
+        <v>-91907</v>
       </c>
       <c r="BA39" s="36" t="n">
         <f aca="false">-[5]Oct!$P$1+[5]Oct!$AM$1</f>
@@ -26776,14 +26776,14 @@
       <c r="BF39" s="54"/>
       <c r="BG39" s="36" t="n">
         <f aca="false">SUM(AV39:BF39)</f>
-        <v>0</v>
+        <v>-780460</v>
       </c>
       <c r="BH39" s="57"/>
       <c r="BI39" s="36"/>
       <c r="BJ39" s="36"/>
       <c r="BK39" s="36" t="n">
         <f aca="false">-[4]Nov!$P$1+[4]Nov!$AM$1</f>
-        <v>0</v>
+        <v>-137960</v>
       </c>
       <c r="BL39" s="36" t="n">
         <f aca="false">-[5]Nov!$P$1+[5]Nov!$AM$1</f>
@@ -26802,14 +26802,14 @@
       <c r="BQ39" s="54"/>
       <c r="BR39" s="36" t="n">
         <f aca="false">SUM(BG39:BQ39)</f>
-        <v>0</v>
+        <v>-918420</v>
       </c>
       <c r="BS39" s="57"/>
       <c r="BT39" s="36"/>
       <c r="BU39" s="36"/>
       <c r="BV39" s="36" t="n">
         <f aca="false">-[4]Dec!$P$1+[4]Dec!$AM$1</f>
-        <v>0</v>
+        <v>-230025</v>
       </c>
       <c r="BW39" s="36" t="n">
         <f aca="false">-[5]Dec!$P$1+[5]Dec!$AM$1</f>
@@ -26828,14 +26828,14 @@
       <c r="CB39" s="54"/>
       <c r="CC39" s="36" t="n">
         <f aca="false">SUM(BR39:CB39)</f>
-        <v>0</v>
+        <v>-1148445</v>
       </c>
       <c r="CD39" s="57"/>
       <c r="CE39" s="36"/>
       <c r="CF39" s="36"/>
       <c r="CG39" s="36" t="n">
         <f aca="false">-[4]Jan!$P$1+[4]Jan!$AM$1</f>
-        <v>0</v>
+        <v>-138138</v>
       </c>
       <c r="CH39" s="36" t="n">
         <f aca="false">-[5]Jan!$P$1+[5]Jan!$AM$1</f>
@@ -26854,14 +26854,14 @@
       <c r="CM39" s="54"/>
       <c r="CN39" s="36" t="n">
         <f aca="false">SUM(CC39:CM39)</f>
-        <v>0</v>
+        <v>-1286583</v>
       </c>
       <c r="CO39" s="57"/>
       <c r="CP39" s="36"/>
       <c r="CQ39" s="36"/>
       <c r="CR39" s="36" t="n">
         <f aca="false">-[4]Feb!$P$1+[4]Feb!$AM$1</f>
-        <v>0</v>
+        <v>-184309</v>
       </c>
       <c r="CS39" s="36" t="n">
         <f aca="false">-[5]Feb!$P$1+[5]Feb!$AM$1</f>
@@ -26880,14 +26880,14 @@
       <c r="CX39" s="54"/>
       <c r="CY39" s="36" t="n">
         <f aca="false">SUM(CN39:CX39)</f>
-        <v>0</v>
+        <v>-1470892</v>
       </c>
       <c r="CZ39" s="57"/>
       <c r="DA39" s="36"/>
       <c r="DB39" s="36"/>
       <c r="DC39" s="36" t="n">
         <f aca="false">-[4]Mar!$P$1+[4]Mar!$AM$1</f>
-        <v>0</v>
+        <v>-138305</v>
       </c>
       <c r="DD39" s="36" t="n">
         <f aca="false">-[5]Mar!$P$1+[5]Mar!$AM$1</f>
@@ -26906,14 +26906,14 @@
       <c r="DI39" s="54"/>
       <c r="DJ39" s="36" t="n">
         <f aca="false">SUM(CY39:DI39)</f>
-        <v>0</v>
+        <v>-1609197</v>
       </c>
       <c r="DK39" s="57"/>
       <c r="DL39" s="36"/>
       <c r="DM39" s="36"/>
       <c r="DN39" s="36" t="n">
         <f aca="false">-[4]Apr!$P$1+[4]Apr!$AM$1</f>
-        <v>0</v>
+        <v>-92271</v>
       </c>
       <c r="DO39" s="36" t="n">
         <f aca="false">-[5]Apr!$P$1+[5]Apr!$AM$1</f>
@@ -26932,14 +26932,14 @@
       <c r="DT39" s="54"/>
       <c r="DU39" s="36" t="n">
         <f aca="false">SUM(DJ39:DT39)</f>
-        <v>0</v>
+        <v>-1701468</v>
       </c>
       <c r="DV39" s="57"/>
       <c r="DW39" s="36"/>
       <c r="DX39" s="36"/>
       <c r="DY39" s="36" t="n">
         <f aca="false">-[4]May!$P$1+[4]May!$AM$1</f>
-        <v>0</v>
+        <v>-184677</v>
       </c>
       <c r="DZ39" s="36" t="n">
         <f aca="false">-[5]May!$P$1+[5]May!$AM$1</f>
@@ -26958,13 +26958,13 @@
       <c r="EE39" s="54"/>
       <c r="EF39" s="36" t="n">
         <f aca="false">SUM(DU39:EE39)</f>
-        <v>0</v>
+        <v>-1886145</v>
       </c>
       <c r="EG39" s="54"/>
       <c r="EI39" s="54"/>
       <c r="EJ39" s="36" t="n">
         <f aca="false">SUM(EF39:EH39)</f>
-        <v>0</v>
+        <v>-1886145</v>
       </c>
       <c r="EK39" s="54"/>
     </row>
@@ -27808,12 +27808,12 @@
       <c r="EG43" s="54"/>
       <c r="EH43" s="36" t="n">
         <f aca="false">-'PubP&amp;L'!F54</f>
-        <v>-217798.7775</v>
+        <v>-223144.7775</v>
       </c>
       <c r="EI43" s="54"/>
       <c r="EJ43" s="36" t="n">
         <f aca="false">SUM(EF43:EH43)</f>
-        <v>-217798.7775</v>
+        <v>-223144.7775</v>
       </c>
       <c r="EK43" s="54"/>
     </row>
@@ -28442,18 +28442,18 @@
       <c r="EC47" s="36"/>
       <c r="ED47" s="36" t="n">
         <f aca="false">CorporationTax!K35</f>
-        <v>51792.3058333333</v>
+        <v>53046.3058333333</v>
       </c>
       <c r="EE47" s="54"/>
       <c r="EF47" s="36" t="n">
         <f aca="false">SUM(DU47:EE47)</f>
-        <v>51792.3058333333</v>
+        <v>53046.3058333333</v>
       </c>
       <c r="EG47" s="54"/>
       <c r="EI47" s="54"/>
       <c r="EJ47" s="36" t="n">
         <f aca="false">SUM(EF47:EH47)</f>
-        <v>51792.3058333333</v>
+        <v>53046.3058333333</v>
       </c>
       <c r="EK47" s="54"/>
     </row>
@@ -28822,12 +28822,12 @@
       <c r="EG49" s="54"/>
       <c r="EH49" s="36" t="n">
         <f aca="false">'PubP&amp;L'!F54</f>
-        <v>217798.7775</v>
+        <v>223144.7775</v>
       </c>
       <c r="EI49" s="54"/>
       <c r="EJ49" s="36" t="n">
         <f aca="false">SUM(EF49:EH49)</f>
-        <v>217798.7775</v>
+        <v>223144.7775</v>
       </c>
       <c r="EK49" s="54"/>
     </row>
@@ -37188,14 +37188,14 @@
       </c>
       <c r="J88" s="36" t="n">
         <f aca="false">-[6]Jun!$Q$1</f>
-        <v>-0</v>
+        <v>-500</v>
       </c>
       <c r="K88" s="36"/>
       <c r="L88" s="36"/>
       <c r="N88" s="57"/>
       <c r="O88" s="36" t="n">
         <f aca="false">SUM(D88:N88)</f>
-        <v>0</v>
+        <v>-500</v>
       </c>
       <c r="P88" s="57"/>
       <c r="Q88" s="36"/>
@@ -37218,7 +37218,7 @@
       <c r="Y88" s="54"/>
       <c r="Z88" s="36" t="n">
         <f aca="false">SUM(O88:Y88)</f>
-        <v>0</v>
+        <v>-500</v>
       </c>
       <c r="AA88" s="57"/>
       <c r="AB88" s="36"/>
@@ -37241,7 +37241,7 @@
       <c r="AJ88" s="54"/>
       <c r="AK88" s="36" t="n">
         <f aca="false">SUM(Z88:AJ88)</f>
-        <v>0</v>
+        <v>-500</v>
       </c>
       <c r="AL88" s="57"/>
       <c r="AM88" s="36"/>
@@ -37256,7 +37256,7 @@
       </c>
       <c r="AQ88" s="36" t="n">
         <f aca="false">-[6]Sep!$Q$1</f>
-        <v>-0</v>
+        <v>-300</v>
       </c>
       <c r="AR88" s="36"/>
       <c r="AS88" s="36"/>
@@ -37264,7 +37264,7 @@
       <c r="AU88" s="54"/>
       <c r="AV88" s="36" t="n">
         <f aca="false">SUM(AK88:AU88)</f>
-        <v>0</v>
+        <v>-800</v>
       </c>
       <c r="AW88" s="57"/>
       <c r="AX88" s="36"/>
@@ -37287,7 +37287,7 @@
       <c r="BF88" s="54"/>
       <c r="BG88" s="36" t="n">
         <f aca="false">SUM(AV88:BF88)</f>
-        <v>0</v>
+        <v>-800</v>
       </c>
       <c r="BH88" s="57"/>
       <c r="BI88" s="36"/>
@@ -37310,7 +37310,7 @@
       <c r="BQ88" s="54"/>
       <c r="BR88" s="36" t="n">
         <f aca="false">SUM(BG88:BQ88)</f>
-        <v>0</v>
+        <v>-800</v>
       </c>
       <c r="BS88" s="57"/>
       <c r="BT88" s="36"/>
@@ -37325,7 +37325,7 @@
       </c>
       <c r="BX88" s="36" t="n">
         <f aca="false">-[6]Dec!$Q$1</f>
-        <v>-0</v>
+        <v>-500</v>
       </c>
       <c r="BY88" s="36"/>
       <c r="BZ88" s="36"/>
@@ -37333,7 +37333,7 @@
       <c r="CB88" s="54"/>
       <c r="CC88" s="36" t="n">
         <f aca="false">SUM(BR88:CB88)</f>
-        <v>0</v>
+        <v>-1300</v>
       </c>
       <c r="CD88" s="57"/>
       <c r="CE88" s="36"/>
@@ -37356,7 +37356,7 @@
       <c r="CM88" s="54"/>
       <c r="CN88" s="36" t="n">
         <f aca="false">SUM(CC88:CM88)</f>
-        <v>0</v>
+        <v>-1300</v>
       </c>
       <c r="CO88" s="57"/>
       <c r="CP88" s="36"/>
@@ -37379,7 +37379,7 @@
       <c r="CX88" s="54"/>
       <c r="CY88" s="36" t="n">
         <f aca="false">SUM(CN88:CX88)</f>
-        <v>0</v>
+        <v>-1300</v>
       </c>
       <c r="CZ88" s="57"/>
       <c r="DA88" s="36"/>
@@ -37394,7 +37394,7 @@
       </c>
       <c r="DE88" s="36" t="n">
         <f aca="false">-[6]Mar!$Q$1</f>
-        <v>-0</v>
+        <v>-300</v>
       </c>
       <c r="DF88" s="36"/>
       <c r="DG88" s="36"/>
@@ -37402,7 +37402,7 @@
       <c r="DI88" s="54"/>
       <c r="DJ88" s="36" t="n">
         <f aca="false">SUM(CY88:DI88)</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="DK88" s="57"/>
       <c r="DL88" s="36"/>
@@ -37425,7 +37425,7 @@
       <c r="DT88" s="54"/>
       <c r="DU88" s="36" t="n">
         <f aca="false">SUM(DJ88:DT88)</f>
-        <v>0</v>
+        <v>-1600</v>
       </c>
       <c r="DV88" s="57"/>
       <c r="DW88" s="36"/>
@@ -37436,7 +37436,7 @@
       </c>
       <c r="DZ88" s="36" t="n">
         <f aca="false">-[5]May!$Q$1</f>
-        <v>-0</v>
+        <v>-5000</v>
       </c>
       <c r="EA88" s="36" t="n">
         <f aca="false">-[6]May!$Q$1</f>
@@ -37448,13 +37448,13 @@
       <c r="EE88" s="54"/>
       <c r="EF88" s="36" t="n">
         <f aca="false">SUM(DU88:EE88)</f>
-        <v>0</v>
+        <v>-6600</v>
       </c>
       <c r="EG88" s="54"/>
       <c r="EI88" s="54"/>
       <c r="EJ88" s="36" t="n">
         <f aca="false">SUM(EF88:EH88)</f>
-        <v>0</v>
+        <v>-6600</v>
       </c>
       <c r="EK88" s="54"/>
     </row>
@@ -37905,7 +37905,7 @@
       </c>
       <c r="H91" s="36" t="n">
         <f aca="false">SUM(H4:H90)</f>
-        <v>0</v>
+        <v>-132637</v>
       </c>
       <c r="I91" s="36" t="n">
         <f aca="false">SUM(I4:I90)</f>
@@ -37917,7 +37917,7 @@
       </c>
       <c r="K91" s="36" t="n">
         <f aca="false">SUM(K4:K90)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="L91" s="36" t="n">
         <f aca="false">SUM(L4:L90)</f>
@@ -37930,7 +37930,7 @@
       <c r="N91" s="54"/>
       <c r="O91" s="36" t="n">
         <f aca="false">SUM(O4:O90)</f>
-        <v>3.09228198602796E-011</v>
+        <v>-132622</v>
       </c>
       <c r="P91" s="54"/>
       <c r="Q91" s="36" t="n">
@@ -37943,7 +37943,7 @@
       </c>
       <c r="S91" s="36" t="n">
         <f aca="false">SUM(S4:S90)</f>
-        <v>0</v>
+        <v>-132286</v>
       </c>
       <c r="T91" s="36" t="n">
         <f aca="false">SUM(T4:T90)</f>
@@ -37951,7 +37951,7 @@
       </c>
       <c r="U91" s="36" t="n">
         <f aca="false">SUM(U4:U90)</f>
-        <v>0</v>
+        <v>-45858</v>
       </c>
       <c r="V91" s="36" t="n">
         <f aca="false">SUM(V4:V90)</f>
@@ -37968,7 +37968,7 @@
       <c r="Y91" s="54"/>
       <c r="Z91" s="36" t="n">
         <f aca="false">SUM(Z4:Z90)</f>
-        <v>6.18456397205591E-011</v>
+        <v>-310766</v>
       </c>
       <c r="AA91" s="54"/>
       <c r="AB91" s="36" t="n">
@@ -37981,7 +37981,7 @@
       </c>
       <c r="AD91" s="36" t="n">
         <f aca="false">SUM(AD4:AD90)</f>
-        <v>0</v>
+        <v>-132684</v>
       </c>
       <c r="AE91" s="36" t="n">
         <f aca="false">SUM(AE4:AE90)</f>
@@ -37989,11 +37989,11 @@
       </c>
       <c r="AF91" s="36" t="n">
         <f aca="false">SUM(AF4:AF90)</f>
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="AG91" s="36" t="n">
         <f aca="false">SUM(AG4:AG90)</f>
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="AH91" s="36" t="n">
         <f aca="false">SUM(AH4:AH90)</f>
@@ -38006,7 +38006,7 @@
       <c r="AJ91" s="54"/>
       <c r="AK91" s="36" t="n">
         <f aca="false">SUM(AK4:AK90)</f>
-        <v>9.45874489843845E-011</v>
+        <v>-443145</v>
       </c>
       <c r="AL91" s="54"/>
       <c r="AM91" s="36" t="n">
@@ -38019,7 +38019,7 @@
       </c>
       <c r="AO91" s="36" t="n">
         <f aca="false">SUM(AO4:AO90)</f>
-        <v>0</v>
+        <v>-224488</v>
       </c>
       <c r="AP91" s="36" t="n">
         <f aca="false">SUM(AP4:AP90)</f>
@@ -38044,7 +38044,7 @@
       <c r="AU91" s="54"/>
       <c r="AV91" s="36" t="n">
         <f aca="false">SUM(AV4:AV90)</f>
-        <v>1.23691279441118E-010</v>
+        <v>-667633</v>
       </c>
       <c r="AW91" s="54"/>
       <c r="AX91" s="36" t="n">
@@ -38057,7 +38057,7 @@
       </c>
       <c r="AZ91" s="36" t="n">
         <f aca="false">SUM(AZ4:AZ90)</f>
-        <v>0</v>
+        <v>-86807</v>
       </c>
       <c r="BA91" s="36" t="n">
         <f aca="false">SUM(BA4:BA90)</f>
@@ -38082,7 +38082,7 @@
       <c r="BF91" s="54"/>
       <c r="BG91" s="36" t="n">
         <f aca="false">SUM(BG4:BG90)</f>
-        <v>1.65982783073559E-010</v>
+        <v>-754440</v>
       </c>
       <c r="BH91" s="54"/>
       <c r="BI91" s="36" t="n">
@@ -38095,7 +38095,7 @@
       </c>
       <c r="BK91" s="36" t="n">
         <f aca="false">SUM(BK4:BK90)</f>
-        <v>0</v>
+        <v>-133360</v>
       </c>
       <c r="BL91" s="36" t="n">
         <f aca="false">SUM(BL4:BL90)</f>
@@ -38107,7 +38107,7 @@
       </c>
       <c r="BN91" s="36" t="n">
         <f aca="false">SUM(BN4:BN90)</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="BO91" s="36" t="n">
         <f aca="false">SUM(BO4:BO90)</f>
@@ -38120,7 +38120,7 @@
       <c r="BQ91" s="54"/>
       <c r="BR91" s="36" t="n">
         <f aca="false">SUM(BR4:BR90)</f>
-        <v>1.95086613530293E-010</v>
+        <v>-887782</v>
       </c>
       <c r="BS91" s="54"/>
       <c r="BT91" s="36" t="n">
@@ -38133,7 +38133,7 @@
       </c>
       <c r="BV91" s="36" t="n">
         <f aca="false">SUM(BV4:BV90)</f>
-        <v>0</v>
+        <v>-188025</v>
       </c>
       <c r="BW91" s="36" t="n">
         <f aca="false">SUM(BW4:BW90)</f>
@@ -38141,7 +38141,7 @@
       </c>
       <c r="BX91" s="36" t="n">
         <f aca="false">SUM(BX4:BX90)</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="BY91" s="36" t="n">
         <f aca="false">SUM(BY4:BY90)</f>
@@ -38158,7 +38158,7 @@
       <c r="CB91" s="54"/>
       <c r="CC91" s="36" t="n">
         <f aca="false">SUM(CC4:CC90)</f>
-        <v>2.38742359215394E-010</v>
+        <v>-1075687</v>
       </c>
       <c r="CD91" s="54"/>
       <c r="CE91" s="36" t="n">
@@ -38171,7 +38171,7 @@
       </c>
       <c r="CG91" s="36" t="n">
         <f aca="false">SUM(CG4:CG90)</f>
-        <v>0</v>
+        <v>-133238</v>
       </c>
       <c r="CH91" s="36" t="n">
         <f aca="false">SUM(CH4:CH90)</f>
@@ -38196,7 +38196,7 @@
       <c r="CM91" s="54"/>
       <c r="CN91" s="36" t="n">
         <f aca="false">SUM(CN4:CN90)</f>
-        <v>2.53294274443761E-010</v>
+        <v>-1208925</v>
       </c>
       <c r="CO91" s="54"/>
       <c r="CP91" s="36" t="n">
@@ -38209,7 +38209,7 @@
       </c>
       <c r="CR91" s="36" t="n">
         <f aca="false">SUM(CR4:CR90)</f>
-        <v>0</v>
+        <v>-179109</v>
       </c>
       <c r="CS91" s="36" t="n">
         <f aca="false">SUM(CS4:CS90)</f>
@@ -38221,7 +38221,7 @@
       </c>
       <c r="CU91" s="36" t="n">
         <f aca="false">SUM(CU4:CU90)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="CV91" s="36" t="n">
         <f aca="false">SUM(CV4:CV90)</f>
@@ -38234,7 +38234,7 @@
       <c r="CX91" s="54"/>
       <c r="CY91" s="36" t="n">
         <f aca="false">SUM(CY4:CY90)</f>
-        <v>2.67846189672127E-010</v>
+        <v>-1387984</v>
       </c>
       <c r="CZ91" s="54"/>
       <c r="DA91" s="36" t="n">
@@ -38247,7 +38247,7 @@
       </c>
       <c r="DC91" s="36" t="n">
         <f aca="false">SUM(DC4:DC90)</f>
-        <v>0</v>
+        <v>-128005</v>
       </c>
       <c r="DD91" s="36" t="n">
         <f aca="false">SUM(DD4:DD90)</f>
@@ -38272,7 +38272,7 @@
       <c r="DI91" s="54"/>
       <c r="DJ91" s="36" t="n">
         <f aca="false">SUM(DJ4:DJ90)</f>
-        <v>2.82398104900494E-010</v>
+        <v>-1515989</v>
       </c>
       <c r="DK91" s="54"/>
       <c r="DL91" s="36" t="n">
@@ -38285,7 +38285,7 @@
       </c>
       <c r="DN91" s="36" t="n">
         <f aca="false">SUM(DN4:DN90)</f>
-        <v>0</v>
+        <v>-86871</v>
       </c>
       <c r="DO91" s="36" t="n">
         <f aca="false">SUM(DO4:DO90)</f>
@@ -38293,7 +38293,7 @@
       </c>
       <c r="DP91" s="36" t="n">
         <f aca="false">SUM(DP4:DP90)</f>
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="DQ91" s="36" t="n">
         <f aca="false">SUM(DQ4:DQ90)</f>
@@ -38310,7 +38310,7 @@
       <c r="DT91" s="54"/>
       <c r="DU91" s="36" t="n">
         <f aca="false">SUM(DU4:DU90)</f>
-        <v>3.04225977743045E-010</v>
+        <v>-1602620</v>
       </c>
       <c r="DV91" s="54"/>
       <c r="DW91" s="36" t="n">
@@ -38323,7 +38323,7 @@
       </c>
       <c r="DY91" s="36" t="n">
         <f aca="false">SUM(DY4:DY90)</f>
-        <v>0</v>
+        <v>-174877</v>
       </c>
       <c r="DZ91" s="36" t="n">
         <f aca="false">SUM(DZ4:DZ90)</f>
@@ -38335,7 +38335,7 @@
       </c>
       <c r="EB91" s="36" t="n">
         <f aca="false">SUM(EB4:EB90)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="EC91" s="36" t="n">
         <f aca="false">SUM(EC4:EC90)</f>
@@ -38348,7 +38348,7 @@
       <c r="EE91" s="54"/>
       <c r="EF91" s="36" t="n">
         <f aca="false">SUM(EF4:EF90)</f>
-        <v>3.18777892971411E-010</v>
+        <v>-1777485</v>
       </c>
       <c r="EG91" s="54"/>
       <c r="EH91" s="36" t="n">
@@ -38358,7 +38358,7 @@
       <c r="EI91" s="54"/>
       <c r="EJ91" s="36" t="n">
         <f aca="false">SUM(EJ4:EJ90)</f>
-        <v>3.18777892971411E-010</v>
+        <v>-1777485</v>
       </c>
       <c r="EK91" s="54"/>
     </row>
@@ -40476,11 +40476,11 @@
       </c>
       <c r="B36" s="71" t="n">
         <f aca="false">SUM(C36:N36)</f>
-        <v>0</v>
+        <v>-6600</v>
       </c>
       <c r="C36" s="72" t="n">
         <f aca="false">TrialBalance!O83+TrialBalance!O88+TrialBalance!O89-0</f>
-        <v>0</v>
+        <v>-500</v>
       </c>
       <c r="D36" s="72" t="n">
         <f aca="false">TrialBalance!Z83+TrialBalance!Z88+TrialBalance!Z89-C36</f>
@@ -40492,7 +40492,7 @@
       </c>
       <c r="F36" s="72" t="n">
         <f aca="false">TrialBalance!AV83+TrialBalance!AV88+TrialBalance!AV89-SUM(C36:E36)</f>
-        <v>0</v>
+        <v>-300</v>
       </c>
       <c r="G36" s="72" t="n">
         <f aca="false">TrialBalance!BG83+TrialBalance!BG88+TrialBalance!BG89-SUM(C36:F36)</f>
@@ -40504,7 +40504,7 @@
       </c>
       <c r="I36" s="72" t="n">
         <f aca="false">TrialBalance!CC83+TrialBalance!CC88+TrialBalance!CC89-SUM(C36:H36)</f>
-        <v>0</v>
+        <v>-500</v>
       </c>
       <c r="J36" s="72" t="n">
         <f aca="false">TrialBalance!CN83+TrialBalance!CN88+TrialBalance!CN89-SUM(C36:I36)</f>
@@ -40516,7 +40516,7 @@
       </c>
       <c r="L36" s="72" t="n">
         <f aca="false">TrialBalance!DJ83+TrialBalance!DJ88+TrialBalance!DJ89-SUM(C36:K36)</f>
-        <v>0</v>
+        <v>-300</v>
       </c>
       <c r="M36" s="72" t="n">
         <f aca="false">TrialBalance!DU83+TrialBalance!DU88+TrialBalance!DU89-SUM(C36:L36)</f>
@@ -40524,7 +40524,7 @@
       </c>
       <c r="N36" s="72" t="n">
         <f aca="false">TrialBalance!EF83+TrialBalance!EF88+TrialBalance!EF89-SUM(C36:M36)</f>
-        <v>0</v>
+        <v>-5000</v>
       </c>
       <c r="O36" s="68"/>
     </row>
@@ -40766,11 +40766,11 @@
       </c>
       <c r="B41" s="71" t="n">
         <f aca="false">SUM(B18:B40)</f>
-        <v>53948.25</v>
+        <v>47348.25</v>
       </c>
       <c r="C41" s="74" t="n">
         <f aca="false">SUM(C18:C40)</f>
-        <v>4226.25</v>
+        <v>3726.25</v>
       </c>
       <c r="D41" s="71" t="n">
         <f aca="false">SUM(D18:D40)</f>
@@ -40782,7 +40782,7 @@
       </c>
       <c r="F41" s="71" t="n">
         <f aca="false">SUM(F18:F40)</f>
-        <v>6590.25</v>
+        <v>6290.25</v>
       </c>
       <c r="G41" s="71" t="n">
         <f aca="false">SUM(G18:G40)</f>
@@ -40794,7 +40794,7 @@
       </c>
       <c r="I41" s="71" t="n">
         <f aca="false">SUM(I18:I40)</f>
-        <v>6240.75</v>
+        <v>5740.75</v>
       </c>
       <c r="J41" s="71" t="n">
         <f aca="false">SUM(J18:J40)</f>
@@ -40806,7 +40806,7 @@
       </c>
       <c r="L41" s="71" t="n">
         <f aca="false">SUM(L18:L40)</f>
-        <v>9129.25</v>
+        <v>8829.25</v>
       </c>
       <c r="M41" s="71" t="n">
         <f aca="false">SUM(M18:M40)</f>
@@ -40814,7 +40814,7 @@
       </c>
       <c r="N41" s="71" t="n">
         <f aca="false">SUM(N18:N40)</f>
-        <v>2877.5</v>
+        <v>-2122.5</v>
       </c>
       <c r="O41" s="68"/>
     </row>
@@ -40841,11 +40841,11 @@
       </c>
       <c r="B43" s="71" t="n">
         <f aca="false">B16-B41</f>
-        <v>269591.083333333</v>
+        <v>276191.083333333</v>
       </c>
       <c r="C43" s="71" t="n">
         <f aca="false">C16-C41</f>
-        <v>22722.0833333333</v>
+        <v>23222.0833333333</v>
       </c>
       <c r="D43" s="71" t="n">
         <f aca="false">D16-D41</f>
@@ -40857,7 +40857,7 @@
       </c>
       <c r="F43" s="71" t="n">
         <f aca="false">F16-F41</f>
-        <v>20574.0833333333</v>
+        <v>20874.0833333333</v>
       </c>
       <c r="G43" s="71" t="n">
         <f aca="false">G16-G41</f>
@@ -40869,7 +40869,7 @@
       </c>
       <c r="I43" s="71" t="n">
         <f aca="false">I16-I41</f>
-        <v>22627.5833333333</v>
+        <v>23127.5833333333</v>
       </c>
       <c r="J43" s="71" t="n">
         <f aca="false">J16-J41</f>
@@ -40881,7 +40881,7 @@
       </c>
       <c r="L43" s="71" t="n">
         <f aca="false">L16-L41</f>
-        <v>19555.0833333333</v>
+        <v>19855.0833333333</v>
       </c>
       <c r="M43" s="71" t="n">
         <f aca="false">M16-M41</f>
@@ -40889,7 +40889,7 @@
       </c>
       <c r="N43" s="71" t="n">
         <f aca="false">N16-N41</f>
-        <v>22406.8333333333</v>
+        <v>27406.8333333333</v>
       </c>
       <c r="O43" s="68"/>
     </row>
@@ -40957,11 +40957,11 @@
       </c>
       <c r="B45" s="71" t="n">
         <f aca="false">B43+B44</f>
-        <v>269591.083333333</v>
+        <v>276191.083333333</v>
       </c>
       <c r="C45" s="71" t="n">
         <f aca="false">C43+C44</f>
-        <v>22722.0833333333</v>
+        <v>23222.0833333333</v>
       </c>
       <c r="D45" s="71" t="n">
         <f aca="false">D43+D44</f>
@@ -40973,7 +40973,7 @@
       </c>
       <c r="F45" s="71" t="n">
         <f aca="false">F43+F44</f>
-        <v>20574.0833333333</v>
+        <v>20874.0833333333</v>
       </c>
       <c r="G45" s="71" t="n">
         <f aca="false">G43+G44</f>
@@ -40985,7 +40985,7 @@
       </c>
       <c r="I45" s="71" t="n">
         <f aca="false">I43+I44</f>
-        <v>22627.5833333333</v>
+        <v>23127.5833333333</v>
       </c>
       <c r="J45" s="71" t="n">
         <f aca="false">J43+J44</f>
@@ -40997,7 +40997,7 @@
       </c>
       <c r="L45" s="71" t="n">
         <f aca="false">L43+L44</f>
-        <v>19555.0833333333</v>
+        <v>19855.0833333333</v>
       </c>
       <c r="M45" s="71" t="n">
         <f aca="false">M43+M44</f>
@@ -41005,7 +41005,7 @@
       </c>
       <c r="N45" s="71" t="n">
         <f aca="false">N43+N44</f>
-        <v>22406.8333333333</v>
+        <v>27406.8333333333</v>
       </c>
       <c r="O45" s="68"/>
     </row>
@@ -41833,7 +41833,7 @@
       <c r="D39" s="88"/>
       <c r="E39" s="86" t="n">
         <f aca="false">TrialBalance!EJ83+TrialBalance!EJ88+TrialBalance!EJ89</f>
-        <v>0</v>
+        <v>-6600</v>
       </c>
       <c r="H39" s="89"/>
       <c r="I39" s="89"/>
@@ -41940,7 +41940,7 @@
       <c r="E44" s="103"/>
       <c r="F44" s="104" t="n">
         <f aca="false">SUM(E21:E43)</f>
-        <v>53948.25</v>
+        <v>47348.25</v>
       </c>
       <c r="H44" s="89"/>
       <c r="I44" s="89"/>
@@ -41976,7 +41976,7 @@
       <c r="E46" s="103"/>
       <c r="F46" s="104" t="n">
         <f aca="false">F18-F44</f>
-        <v>269591.083333333</v>
+        <v>276191.083333333</v>
       </c>
       <c r="H46" s="89"/>
       <c r="I46" s="89"/>
@@ -42031,7 +42031,7 @@
       <c r="E49" s="103"/>
       <c r="F49" s="104" t="n">
         <f aca="false">F46+F48</f>
-        <v>269591.083333333</v>
+        <v>276191.083333333</v>
       </c>
       <c r="H49" s="89"/>
       <c r="I49" s="89"/>
@@ -42052,7 +42052,7 @@
       <c r="D50" s="101"/>
       <c r="F50" s="86" t="n">
         <f aca="false">TrialBalance!EJ47</f>
-        <v>51792.3058333333</v>
+        <v>53046.3058333333</v>
       </c>
       <c r="H50" s="89"/>
       <c r="I50" s="89"/>
@@ -42075,7 +42075,7 @@
       <c r="E51" s="103"/>
       <c r="F51" s="104" t="n">
         <f aca="false">F49-F50</f>
-        <v>217798.7775</v>
+        <v>223144.7775</v>
       </c>
       <c r="H51" s="89"/>
       <c r="I51" s="89"/>
@@ -42136,7 +42136,7 @@
       </c>
       <c r="F54" s="104" t="n">
         <f aca="false">F51-F52</f>
-        <v>217798.7775</v>
+        <v>223144.7775</v>
       </c>
       <c r="H54" s="89"/>
       <c r="I54" s="89"/>
@@ -42313,7 +42313,7 @@
       </c>
       <c r="E11" s="115" t="n">
         <f aca="false">TrialBalance!EJ20</f>
-        <v>424900</v>
+        <v>226300</v>
       </c>
       <c r="F11" s="115"/>
     </row>
@@ -42328,7 +42328,7 @@
       </c>
       <c r="E12" s="119" t="n">
         <f aca="false">IF(SUM(TrialBalance!EJ22:EJ24)&gt;0,SUM(TrialBalance!EJ22:EJ24)+TrialBalance!EJ25+TrialBalance!EJ26,TrialBalance!EJ25)</f>
-        <v>0</v>
+        <v>318135</v>
       </c>
       <c r="F12" s="115"/>
     </row>
@@ -42344,7 +42344,7 @@
       <c r="D13" s="117"/>
       <c r="E13" s="116" t="n">
         <f aca="false">SUM(E10:E12)</f>
-        <v>424900</v>
+        <v>544435</v>
       </c>
       <c r="F13" s="118"/>
     </row>
@@ -42390,7 +42390,7 @@
       </c>
       <c r="E17" s="115" t="n">
         <f aca="false">-TrialBalance!EJ35</f>
-        <v>51792.3058333333</v>
+        <v>53046.3058333333</v>
       </c>
       <c r="F17" s="115"/>
     </row>
@@ -42405,7 +42405,7 @@
       </c>
       <c r="E18" s="115" t="n">
         <f aca="false">-SUM(TrialBalance!EJ32:EJ34)</f>
-        <v>70816.6666666667</v>
+        <v>75091.6666666667</v>
       </c>
       <c r="F18" s="115"/>
     </row>
@@ -42438,7 +42438,7 @@
       <c r="D20" s="117"/>
       <c r="E20" s="116" t="n">
         <f aca="false">SUM(E16:E19)</f>
-        <v>233601.2225</v>
+        <v>239130.2225</v>
       </c>
       <c r="F20" s="118"/>
       <c r="G20" s="120"/>
@@ -42465,7 +42465,7 @@
       <c r="E22" s="118"/>
       <c r="F22" s="116" t="n">
         <f aca="false">E13-E20</f>
-        <v>191298.7775</v>
+        <v>305304.7775</v>
       </c>
       <c r="G22" s="120"/>
     </row>
@@ -42518,7 +42518,7 @@
       <c r="E26" s="118"/>
       <c r="F26" s="116" t="n">
         <f aca="false">SUM(F6:F25)</f>
-        <v>217798.7775</v>
+        <v>331804.7775</v>
       </c>
       <c r="G26" s="120"/>
     </row>
@@ -42551,7 +42551,7 @@
       <c r="D29" s="88"/>
       <c r="E29" s="115" t="n">
         <f aca="false">-TrialBalance!EJ39</f>
-        <v>-0</v>
+        <v>1886145</v>
       </c>
       <c r="F29" s="115"/>
       <c r="G29" s="87"/>
@@ -42584,7 +42584,7 @@
       <c r="E31" s="115"/>
       <c r="F31" s="116" t="n">
         <f aca="false">SUM(E29:E30)</f>
-        <v>0</v>
+        <v>1886145</v>
       </c>
     </row>
     <row r="32" s="120" customFormat="true" ht="12" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -42614,7 +42614,7 @@
       </c>
       <c r="F33" s="116" t="n">
         <f aca="false">F26-F31</f>
-        <v>217798.7775</v>
+        <v>-1554340.2225</v>
       </c>
       <c r="G33" s="120"/>
     </row>
@@ -42664,7 +42664,7 @@
       <c r="E37" s="115"/>
       <c r="F37" s="115" t="n">
         <f aca="false">-TrialBalance!EJ43</f>
-        <v>217798.7775</v>
+        <v>223144.7775</v>
       </c>
       <c r="G37" s="87"/>
       <c r="O37" s="87"/>
@@ -42704,7 +42704,7 @@
       </c>
       <c r="F39" s="116" t="n">
         <f aca="false">SUM(F36:F38)</f>
-        <v>217798.7775</v>
+        <v>223144.7775</v>
       </c>
       <c r="G39" s="120"/>
     </row>
@@ -43466,7 +43466,7 @@
       <c r="C41" s="137"/>
       <c r="D41" s="136" t="n">
         <f aca="false">CorporationTax!K35</f>
-        <v>51792.3058333333</v>
+        <v>53046.3058333333</v>
       </c>
       <c r="G41" s="89"/>
     </row>
@@ -44437,7 +44437,7 @@
       <c r="J5" s="178"/>
       <c r="K5" s="191" t="n">
         <f aca="false">'PubP&amp;L'!F46</f>
-        <v>269591.083333333</v>
+        <v>276191.083333333</v>
       </c>
       <c r="L5" s="185"/>
     </row>
@@ -44555,7 +44555,7 @@
       <c r="J12" s="178"/>
       <c r="K12" s="191" t="n">
         <f aca="false">K5+K10</f>
-        <v>272591.083333333</v>
+        <v>279191.083333333</v>
       </c>
       <c r="L12" s="185"/>
     </row>
@@ -44765,7 +44765,7 @@
       <c r="J22" s="178"/>
       <c r="K22" s="209" t="n">
         <f aca="false">K12-K20</f>
-        <v>272591.083333333</v>
+        <v>279191.083333333</v>
       </c>
       <c r="L22" s="185"/>
     </row>
@@ -44867,7 +44867,7 @@
       <c r="J28" s="178"/>
       <c r="K28" s="209" t="n">
         <f aca="false">K22+K24-K26</f>
-        <v>272591.083333333</v>
+        <v>279191.083333333</v>
       </c>
       <c r="L28" s="185"/>
     </row>
@@ -44965,7 +44965,7 @@
       </c>
       <c r="F33" s="186" t="n">
         <f aca="false">IF(K28&gt;0,K28*A33/A35,0)</f>
-        <v>136109.090857273</v>
+        <v>139404.576493388</v>
       </c>
       <c r="G33" s="224" t="n">
         <f aca="false">Admin!P6</f>
@@ -44974,7 +44974,7 @@
       <c r="H33" s="224"/>
       <c r="I33" s="225" t="n">
         <f aca="false">F33*G33/100</f>
-        <v>25860.7272628819</v>
+        <v>26486.8695337437</v>
       </c>
       <c r="J33" s="226"/>
       <c r="K33" s="178"/>
@@ -45002,7 +45002,7 @@
       </c>
       <c r="F34" s="186" t="n">
         <f aca="false">IF(K28&gt;0,K28*A34/A35,0)</f>
-        <v>136481.99247606</v>
+        <v>139786.506839945</v>
       </c>
       <c r="G34" s="224" t="n">
         <f aca="false">Admin!P7</f>
@@ -45011,7 +45011,7 @@
       <c r="H34" s="224"/>
       <c r="I34" s="225" t="n">
         <f aca="false">F34*G34/100</f>
-        <v>25931.5785704514</v>
+        <v>26559.4362995896</v>
       </c>
       <c r="J34" s="226"/>
       <c r="K34" s="178"/>
@@ -45035,7 +45035,7 @@
       <c r="J35" s="227"/>
       <c r="K35" s="228" t="n">
         <f aca="false">SUM(I33:I34)</f>
-        <v>51792.3058333333</v>
+        <v>53046.3058333333</v>
       </c>
       <c r="L35" s="185"/>
     </row>
@@ -45101,7 +45101,7 @@
       <c r="J39" s="178"/>
       <c r="K39" s="232" t="n">
         <f aca="false">K35-K37</f>
-        <v>51792.3058333333</v>
+        <v>53046.3058333333</v>
       </c>
       <c r="L39" s="185"/>
     </row>
@@ -49954,7 +49954,7 @@
       </c>
       <c r="Z70" s="302" t="n">
         <f aca="false">IF(CorporationTax!K22&gt;0,CorporationTax!K22," ")</f>
-        <v>272591.083333333</v>
+        <v>279191.083333333</v>
       </c>
       <c r="AA70" s="302"/>
       <c r="AB70" s="302"/>
@@ -50172,7 +50172,7 @@
       </c>
       <c r="AJ74" s="302" t="n">
         <f aca="false">SUM(Z69:AF70)-SUM(Z72:AF73)</f>
-        <v>272591.083333333</v>
+        <v>279191.083333333</v>
       </c>
       <c r="AK74" s="302"/>
       <c r="AL74" s="302"/>
@@ -51070,7 +51070,7 @@
       </c>
       <c r="AJ92" s="302" t="n">
         <f aca="false">IF(AJ74&gt;0,AJ74+SUM(AJ76:AJ80)+AJ88,0)</f>
-        <v>272591.083333333</v>
+        <v>279191.083333333</v>
       </c>
       <c r="AK92" s="302"/>
       <c r="AL92" s="302"/>
@@ -51955,7 +51955,7 @@
       </c>
       <c r="AJ110" s="302" t="n">
         <f aca="false">AJ92-Z96-Z98-Z104-Z106</f>
-        <v>272591.083333333</v>
+        <v>279191.083333333</v>
       </c>
       <c r="AK110" s="302"/>
       <c r="AL110" s="302"/>
@@ -52733,7 +52733,7 @@
       </c>
       <c r="N126" s="328" t="n">
         <f aca="false">CorporationTax!F33</f>
-        <v>136109.090857273</v>
+        <v>139404.576493388</v>
       </c>
       <c r="O126" s="328"/>
       <c r="P126" s="328"/>
@@ -52767,7 +52767,7 @@
       </c>
       <c r="AJ126" s="330" t="n">
         <f aca="false">CorporationTax!I33</f>
-        <v>25860.7272628819</v>
+        <v>26486.8695337437</v>
       </c>
       <c r="AK126" s="330"/>
       <c r="AL126" s="330"/>
@@ -53026,7 +53026,7 @@
       </c>
       <c r="AJ131" s="330" t="n">
         <f aca="false">AJ126+AJ128</f>
-        <v>25860.7272628819</v>
+        <v>26486.8695337437</v>
       </c>
       <c r="AK131" s="330"/>
       <c r="AL131" s="330"/>
@@ -53742,7 +53742,7 @@
       </c>
       <c r="AJ145" s="330" t="n">
         <f aca="false">AJ131</f>
-        <v>25860.7272628819</v>
+        <v>26486.8695337437</v>
       </c>
       <c r="AK145" s="330"/>
       <c r="AL145" s="330"/>
@@ -54444,7 +54444,7 @@
       </c>
       <c r="AJ159" s="330" t="n">
         <f aca="false">IF(AJ145&gt;0,AJ145+AJ149-AJ154,0)</f>
-        <v>25860.7272628819</v>
+        <v>26486.8695337437</v>
       </c>
       <c r="AK159" s="330"/>
       <c r="AL159" s="330"/>
@@ -54793,7 +54793,7 @@
       </c>
       <c r="AJ166" s="330" t="n">
         <f aca="false">IF(AJ159&gt;0,AJ159-AJ163,0)</f>
-        <v>25860.7272628819</v>
+        <v>26486.8695337437</v>
       </c>
       <c r="AK166" s="330"/>
       <c r="AL166" s="330"/>

</xml_diff>